<commit_message>
Review fixes: VIN monitor linearity and reset, full-scale summary, design notes
- U18 inputs swapped (IN+ = OVP_DIV, IN- = RAMP via R109 1k); R110 4.7M
  hysteresis now on the divider, not the ramp (old 1M path bent the ramp:
  +12.5 % error at 12 V; now < 0.02 % in simulation)
- Reset pulse hardened: C81 220p C0G, R107 100k so C82 always fully discharges
- OVP trip corrected to 50.26 V rising / 49.83 V falling; TL431A noted as 1 %
- PCB re-routed locally, values synced to schematic; DRC clean, parity OK,
  isolation 4.0 mm
- Design notes: full-scale and threshold summary, VIN monitor firmware formula
  and two-point calibration; exported to DOCX and PDF
- Pin-map, BOM, Gerbers, CPL, EasyEDA zip and PDFs regenerated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A35wrnwFKLPSaRSxxHs471
</commit_message>
<xml_diff>
--- a/01_hardware/docs/pin-map.xlsx
+++ b/01_hardware/docs/pin-map.xlsx
@@ -1870,7 +1870,7 @@
       </c>
       <c r="J15" s="8" t="inlineStr">
         <is>
-          <t>Rev D: isolated VIN monitor. Primary ramp/comparator PWM (~200 Hz) through U12 VI2-&gt;VO2; 10k pull-down (R93). VIN = 50.36 V x (T_ramp - t_high) / T_ramp, T_ramp = period - ~20 us; monitor only</t>
+          <t>Rev D: isolated VIN monitor. Primary ramp/comparator PWM (~200 Hz) through U12 VI2-&gt;VO2; 10k pull-down (R93). High while ramp &lt; divider. VIN = 50.47 V x (t_high - t_reset) / (period - t_reset) - 0.20 V, t_reset ~20 us; 2-point calibration; monitor only</t>
         </is>
       </c>
       <c r="K15" s="4" t="inlineStr">
@@ -5333,7 +5333,7 @@
       </c>
       <c r="J52" s="8" t="inlineStr">
         <is>
-          <t>Rev D: primary input OVP, LMV331 + TL431 trip 50.2 V, through U12 VI1-&gt;VO1; high = over-voltage. Configure FLT2 active-high so the HRTIM shuts all outputs in hardware</t>
+          <t>Rev D: primary input OVP, LMV331 + TL431 trip 50.26 V rising / 49.83 V falling, through U12 VI1-&gt;VO1; high = over-voltage. Configure FLT2 active-high so the HRTIM shuts all outputs in hardware</t>
         </is>
       </c>
       <c r="K52" s="4" t="inlineStr">

</xml_diff>

<commit_message>
External REF3030 ADC reference; full review and documentation update
- U19 REF3030AIDBZR (3.000 V +/-0.2 %, LCSC C38423) + C85 drive VREF+ (new net
  VREF_ADC); VREF+ separated from VDDA; R25 (IL zero) and R29 (NTC pull-up)
  moved to VREF_ADC so those channels are ratiometric
- Full scales: VBUS/VOUT 61.8 V, IL +/-18.75 A, IOUT 6.0 A, DAC/COMP 0-3.0 V
- PCB: U19/C85 placed and routed, pins 28/29 hand-routed; DRC clean, parity
  OK, isolation 4.0 mm
- Design notes (DOCX/PDF), root and firmware READMEs, pin-map, layout review
  image, BOM, Gerbers, CPL, EasyEDA zip and PDFs updated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A35wrnwFKLPSaRSxxHs471
</commit_message>
<xml_diff>
--- a/01_hardware/docs/pin-map.xlsx
+++ b/01_hardware/docs/pin-map.xlsx
@@ -1672,7 +1672,7 @@
       </c>
       <c r="J13" s="8" t="inlineStr">
         <is>
-          <t>VBUS divider 100k/5.1k, 1 nF -&gt; 68 V full scale</t>
+          <t>VBUS divider 100k/5.1k 0.1 %, 1 nF -&gt; 61.8 V full scale (VREF+ 3.0 V)</t>
         </is>
       </c>
       <c r="K13" s="4" t="inlineStr">
@@ -1775,7 +1775,7 @@
       </c>
       <c r="J14" s="8" t="inlineStr">
         <is>
-          <t>INA181A2 on 10 mOhm (RSH1): 0.5 V/A, 1k + 10 nF filter</t>
+          <t>INA181A2 on 10 mOhm (RSH1): 0.5 V/A, FS 6.0 A, 1k + 10 nF filter</t>
         </is>
       </c>
       <c r="K14" s="4" t="inlineStr">
@@ -2396,7 +2396,7 @@
       </c>
       <c r="J21" s="8" t="inlineStr">
         <is>
-          <t>NTC 10k B3950 / 10k divider (Rev D: moved from PA4 to PA6)</t>
+          <t>NTC 10k B3950 / 10k pull-up from VREF+ (ratiometric); Rev D: moved from PA4 to PA6</t>
         </is>
       </c>
       <c r="K21" s="4" t="inlineStr">
@@ -2796,7 +2796,7 @@
       </c>
       <c r="J25" s="8" t="inlineStr">
         <is>
-          <t>Inductor current (INA181A1 on 4 mOhm, 1.65 V + 0.08 V/A): buck-mode negative OCP, COMP4 output inverted -&gt; HRTIM fault</t>
+          <t>Inductor current (INA181A1 on 4 mOhm, 1.50 V + 0.08 V/A, +/-18.75 A): buck-mode negative OCP, COMP4 output inverted -&gt; HRTIM fault</t>
         </is>
       </c>
       <c r="K25" s="4" t="inlineStr">
@@ -3119,46 +3119,50 @@
       <c r="AA28" s="4" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="n">
+      <c r="A29" s="7" t="n">
         <v>28</v>
       </c>
-      <c r="B29" s="3" t="inlineStr">
+      <c r="B29" s="8" t="inlineStr">
         <is>
           <t>VREF+</t>
         </is>
       </c>
-      <c r="C29" s="2" t="inlineStr">
+      <c r="C29" s="7" t="inlineStr">
         <is>
           <t>MonoIO</t>
         </is>
       </c>
-      <c r="D29" s="3" t="inlineStr">
-        <is>
-          <t>+3V3A</t>
-        </is>
-      </c>
-      <c r="E29" s="2" t="inlineStr">
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>VREF_ADC</t>
+        </is>
+      </c>
+      <c r="E29" s="7" t="inlineStr">
+        <is>
+          <t>Used</t>
+        </is>
+      </c>
+      <c r="F29" s="9" t="inlineStr">
+        <is>
+          <t>VREF+ input</t>
+        </is>
+      </c>
+      <c r="G29" s="9" t="inlineStr">
         <is>
           <t>Power</t>
         </is>
       </c>
-      <c r="F29" s="3" t="inlineStr">
-        <is>
-          <t>VREF+ input</t>
-        </is>
-      </c>
-      <c r="G29" s="3" t="inlineStr">
-        <is>
-          <t>Power</t>
-        </is>
-      </c>
-      <c r="H29" s="2" t="inlineStr">
+      <c r="H29" s="7" t="inlineStr">
         <is>
           <t>Supply</t>
         </is>
       </c>
-      <c r="I29" s="3" t="inlineStr"/>
-      <c r="J29" s="3" t="inlineStr">
+      <c r="I29" s="8" t="inlineStr">
+        <is>
+          <t>C36.1, C37.1, R25.1, R29.1, U19.2</t>
+        </is>
+      </c>
+      <c r="J29" s="8" t="inlineStr">
         <is>
           <t>Tied to +3V3A (VREFBUF disabled); ADC/DAC full scale = 3.3 V</t>
         </is>
@@ -3211,7 +3215,7 @@
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>Analog supply / reference</t>
+          <t>Analog supply</t>
         </is>
       </c>
       <c r="G30" s="3" t="inlineStr">
@@ -3227,7 +3231,7 @@
       <c r="I30" s="3" t="inlineStr"/>
       <c r="J30" s="3" t="inlineStr">
         <is>
-          <t>VDDA and VREF+ from +3V3 via FB1; VREFBUF off, VREF+ used as input (1 uF + 100 nF)</t>
+          <t>VDDA from +3V3 via FB1 (1 uF + 100 nF); also feeds the REF3030 ADC reference U19</t>
         </is>
       </c>
       <c r="K30" s="4" t="inlineStr"/>
@@ -3523,7 +3527,7 @@
       </c>
       <c r="J34" s="8" t="inlineStr">
         <is>
-          <t>VOUT divider 100k/5.1k; COMP6 = fast hardware OVP (threshold from DAC3)</t>
+          <t>VOUT divider 100k/5.1k 0.1 %, FS 61.8 V; COMP6 = fast hardware OVP (threshold from DAC3)</t>
         </is>
       </c>
       <c r="K34" s="4" t="inlineStr">

</xml_diff>